<commit_message>
Evidence: eliminate 画面HC mis-capture/missing (screen-aware queue, AY/AZ return routes)
</commit_message>
<xml_diff>
--- a/evidence/index.xlsx
+++ b/evidence/index.xlsx
@@ -623,10 +623,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>0</v>
@@ -635,7 +635,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -755,10 +755,10 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>0</v>
@@ -767,7 +767,7 @@
         <v>1</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -818,13 +818,13 @@
         <v>2</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>0</v>
@@ -833,7 +833,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -5009,10 +5009,10 @@
         <v>9</v>
       </c>
       <c r="D138" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E138" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F138" s="2" t="n">
         <v>0</v>
@@ -5243,10 +5243,10 @@
         <v>1</v>
       </c>
       <c r="E145" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F145" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G145" s="2" t="n">
         <v>0</v>
@@ -5255,7 +5255,7 @@
         <v>0</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -5276,10 +5276,10 @@
         <v>1</v>
       </c>
       <c r="E146" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F146" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G146" s="2" t="n">
         <v>0</v>
@@ -5288,7 +5288,7 @@
         <v>0</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -5306,10 +5306,10 @@
         <v>17</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E147" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F147" s="2" t="n">
         <v>0</v>
@@ -5339,10 +5339,10 @@
         <v>17</v>
       </c>
       <c r="D148" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E148" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F148" s="2" t="n">
         <v>0</v>
@@ -5372,10 +5372,10 @@
         <v>17</v>
       </c>
       <c r="D149" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E149" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F149" s="2" t="n">
         <v>0</v>
@@ -5405,10 +5405,10 @@
         <v>17</v>
       </c>
       <c r="D150" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E150" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F150" s="2" t="n">
         <v>0</v>
@@ -6692,10 +6692,10 @@
         <v>4</v>
       </c>
       <c r="D189" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E189" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F189" s="2" t="n">
         <v>0</v>
@@ -6857,10 +6857,10 @@
         <v>4</v>
       </c>
       <c r="D194" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E194" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F194" s="2" t="n">
         <v>0</v>
@@ -7946,10 +7946,10 @@
         <v>25</v>
       </c>
       <c r="D227" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E227" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F227" s="2" t="n">
         <v>0</v>
@@ -8045,22 +8045,22 @@
         <v>2</v>
       </c>
       <c r="D230" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E230" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G230" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I230" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="E230" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F230" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G230" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H230" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I230" s="2" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="231">
@@ -8144,10 +8144,10 @@
         <v>2</v>
       </c>
       <c r="D233" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E233" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F233" s="2" t="n">
         <v>0</v>
@@ -9167,13 +9167,13 @@
         <v>7</v>
       </c>
       <c r="D264" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E264" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F264" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G264" s="2" t="n">
         <v>0</v>
@@ -9182,7 +9182,7 @@
         <v>3</v>
       </c>
       <c r="I264" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="265">
@@ -9200,13 +9200,13 @@
         <v>7</v>
       </c>
       <c r="D265" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E265" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F265" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G265" s="2" t="n">
         <v>0</v>
@@ -9215,7 +9215,7 @@
         <v>3</v>
       </c>
       <c r="I265" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="266">
@@ -9236,10 +9236,10 @@
         <v>1</v>
       </c>
       <c r="E266" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F266" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G266" s="2" t="n">
         <v>0</v>
@@ -9248,7 +9248,7 @@
         <v>1</v>
       </c>
       <c r="I266" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="267">
@@ -9266,13 +9266,13 @@
         <v>4</v>
       </c>
       <c r="D267" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E267" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F267" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G267" s="2" t="n">
         <v>0</v>
@@ -9281,7 +9281,7 @@
         <v>1</v>
       </c>
       <c r="I267" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="268">
@@ -9302,10 +9302,10 @@
         <v>1</v>
       </c>
       <c r="E268" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F268" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G268" s="2" t="n">
         <v>0</v>
@@ -9314,7 +9314,7 @@
         <v>1</v>
       </c>
       <c r="I268" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="269">
@@ -9332,13 +9332,13 @@
         <v>4</v>
       </c>
       <c r="D269" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E269" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F269" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G269" s="2" t="n">
         <v>0</v>
@@ -9347,7 +9347,7 @@
         <v>1</v>
       </c>
       <c r="I269" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="270">
@@ -9434,10 +9434,10 @@
         <v>1</v>
       </c>
       <c r="E272" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F272" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G272" s="2" t="n">
         <v>0</v>
@@ -9446,7 +9446,7 @@
         <v>1</v>
       </c>
       <c r="I272" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="273">
@@ -9497,13 +9497,13 @@
         <v>2</v>
       </c>
       <c r="D274" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E274" s="2" t="n">
         <v>0</v>
       </c>
       <c r="F274" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G274" s="2" t="n">
         <v>0</v>
@@ -9512,7 +9512,7 @@
         <v>0</v>
       </c>
       <c r="I274" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="275">
@@ -9728,10 +9728,10 @@
         <v>10</v>
       </c>
       <c r="D281" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E281" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F281" s="2" t="n">
         <v>0</v>
@@ -9794,10 +9794,10 @@
         <v>4</v>
       </c>
       <c r="D283" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E283" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F283" s="2" t="n">
         <v>0</v>
@@ -9926,10 +9926,10 @@
         <v>4</v>
       </c>
       <c r="D287" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E287" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F287" s="2" t="n">
         <v>0</v>
@@ -10091,10 +10091,10 @@
         <v>7</v>
       </c>
       <c r="D292" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E292" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F292" s="2" t="n">
         <v>0</v>
@@ -10718,10 +10718,10 @@
         <v>4</v>
       </c>
       <c r="D311" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E311" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F311" s="2" t="n">
         <v>0</v>
@@ -10751,10 +10751,10 @@
         <v>4</v>
       </c>
       <c r="D312" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E312" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F312" s="2" t="n">
         <v>0</v>
@@ -10784,10 +10784,10 @@
         <v>4</v>
       </c>
       <c r="D313" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E313" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F313" s="2" t="n">
         <v>0</v>
@@ -10817,10 +10817,10 @@
         <v>4</v>
       </c>
       <c r="D314" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E314" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F314" s="2" t="n">
         <v>0</v>
@@ -10850,10 +10850,10 @@
         <v>4</v>
       </c>
       <c r="D315" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E315" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F315" s="2" t="n">
         <v>0</v>
@@ -11279,10 +11279,10 @@
         <v>7</v>
       </c>
       <c r="D328" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E328" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F328" s="2" t="n">
         <v>0</v>
@@ -14546,10 +14546,10 @@
         <v>4</v>
       </c>
       <c r="D427" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E427" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F427" s="2" t="n">
         <v>0</v>
@@ -15338,10 +15338,10 @@
         <v>10</v>
       </c>
       <c r="D451" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E451" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F451" s="2" t="n">
         <v>0</v>

</xml_diff>